<commit_message>
Atualização automática de preços de eletricidade
</commit_message>
<xml_diff>
--- a/output/spot_price_dailyHour_PT.xlsx
+++ b/output/spot_price_dailyHour_PT.xlsx
@@ -647,82 +647,82 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
       <c r="B2" t="n">
-        <v>200.75</v>
+        <v>216.34</v>
       </c>
       <c r="C2" t="n">
-        <v>194.28</v>
+        <v>209.23</v>
       </c>
       <c r="D2" t="n">
-        <v>192.36</v>
+        <v>203.11</v>
       </c>
       <c r="E2" t="n">
-        <v>180.95</v>
+        <v>200.36</v>
       </c>
       <c r="F2" t="n">
-        <v>170.83</v>
+        <v>202.66</v>
       </c>
       <c r="G2" t="n">
-        <v>180.95</v>
+        <v>207.69</v>
       </c>
       <c r="H2" t="n">
-        <v>187.02</v>
+        <v>229.87</v>
       </c>
       <c r="I2" t="n">
-        <v>190.23</v>
+        <v>255.03</v>
       </c>
       <c r="J2" t="n">
-        <v>164.61</v>
+        <v>264.64</v>
       </c>
       <c r="K2" t="n">
-        <v>77.58</v>
+        <v>212.59</v>
       </c>
       <c r="L2" t="n">
-        <v>0.32</v>
+        <v>127.21</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.14</v>
+        <v>59.82</v>
       </c>
       <c r="N2" t="n">
-        <v>-0.28</v>
+        <v>44.53</v>
       </c>
       <c r="O2" t="n">
-        <v>0</v>
+        <v>47.51</v>
       </c>
       <c r="P2" t="n">
-        <v>-0.01</v>
+        <v>49.15</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.01</v>
+        <v>62</v>
       </c>
       <c r="R2" t="n">
-        <v>0</v>
+        <v>80.56</v>
       </c>
       <c r="S2" t="n">
-        <v>0.48</v>
+        <v>114.2</v>
       </c>
       <c r="T2" t="n">
-        <v>77.78</v>
+        <v>181.34</v>
       </c>
       <c r="U2" t="n">
-        <v>191.49</v>
+        <v>246.08</v>
       </c>
       <c r="V2" t="n">
-        <v>233.83</v>
+        <v>296.25</v>
       </c>
       <c r="W2" t="n">
-        <v>232.37</v>
+        <v>279.12</v>
       </c>
       <c r="X2" t="n">
-        <v>227.46</v>
+        <v>245.96</v>
       </c>
       <c r="Y2" t="n">
-        <v>210.59</v>
+        <v>224.38</v>
       </c>
       <c r="Z2" t="n">
-        <v>121.39</v>
+        <v>177.48</v>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="AB2" t="n">
-        <v>226.06</v>
+        <v>261.43</v>
       </c>
       <c r="AC2" t="inlineStr">
         <is>
@@ -738,19 +738,19 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>233.1</v>
+        <v>287.68</v>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>22h-24h</t>
+          <t>6h-8h</t>
         </is>
       </c>
       <c r="AF2" t="n">
-        <v>219.02</v>
+        <v>242.45</v>
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>9h-18h</t>
+          <t>10h-17h</t>
         </is>
       </c>
     </row>

</xml_diff>